<commit_message>
Initialised new test cases for probelms
</commit_message>
<xml_diff>
--- a/temp_benchmark_data.xlsx
+++ b/temp_benchmark_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\megha\Managing data for minor\Major\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ABDAAD8-5A95-4AEB-81E4-9DE5E5A9B546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD008A7-9933-4F64-B86E-A54F225DEB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="146">
   <si>
     <t>SrNo</t>
   </si>
@@ -525,9 +525,6 @@
     <t>Course Schedule</t>
   </si>
   <si>
-    <t>Determine if all courses can be finished given prerequisites.</t>
-  </si>
-  <si>
     <t>class Solution:
     def canFinish(self, numCourses: int, prerequisites: List[List[int]]) -&gt; bool:
         adj=[[] for _ in range(numCourses)]
@@ -548,9 +545,6 @@
   </si>
   <si>
     <t>Snakes and Ladders</t>
-  </si>
-  <si>
-    <t>Find the shortest path to reach the last square.</t>
   </si>
   <si>
     <t>from collections import deque
@@ -585,9 +579,6 @@
   </si>
   <si>
     <t>Word Ladder</t>
-  </si>
-  <si>
-    <t>Find the shortest transformation sequence from start to end word.</t>
   </si>
   <si>
     <t>from collections import deque
@@ -648,9 +639,6 @@
     <t>Find Minimum in Rotated Sorted Array</t>
   </si>
   <si>
-    <t>Find the minimum element in a rotated sorted array.</t>
-  </si>
-  <si>
     <t xml:space="preserve">class Solution:
     def findMin(self, nums: List[int]) -&gt; int:
         start = 0
@@ -668,9 +656,6 @@
   </si>
   <si>
     <t>Search a 2D Matrix</t>
-  </si>
-  <si>
-    <t>Search for a target in a matrix.</t>
   </si>
   <si>
     <t>class Solution:
@@ -1600,6 +1585,128 @@
   <si>
     <t>class Solution:
     def rightSideView(self, root: Optional[TreeNode]) -&gt; List[int]:</t>
+  </si>
+  <si>
+    <t>There are a total of numCourses courses you have to take, labeled from 0 to numCourses - 1. You are given an array prerequisites where prerequisites[i] = [ai, bi] indicates that you must take course bi first if you want to take course ai.
+For example, the pair [0, 1], indicates that to take course 0 you have to first take course 1.
+Return true if you can finish all courses. Otherwise, return false.
+Example 1:
+Input: numCourses = 2, prerequisites = [[1,0]]
+Output: true
+Explanation: There are a total of 2 courses to take. 
+To take course 1 you should have finished course 0. So it is possible.
+Example 2:
+Input: numCourses = 2, prerequisites = [[1,0],[0,1]]
+Output: false
+Explanation: There are a total of 2 courses to take. 
+To take course 1 you should have finished course 0, and to take course 0 you should also have finished course 1. So it is impossible.
+Constraints:
+1 &lt;= numCourses &lt;= 2000
+0 &lt;= prerequisites.length &lt;= 5000
+prerequisites[i].length == 2
+0 &lt;= ai, bi &lt; numCourses
+All the pairs prerequisites[i] are unique.</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def canFinish(self, numCourses: int, prerequisites: List[List[int]]) -&gt; bool:</t>
+  </si>
+  <si>
+    <t>You are given an n x n integer matrix board where the cells are labeled from 1 to n2 in a Boustrophedon style starting from the bottom left of the board (i.e. board[n - 1][0]) and alternating direction each row.
+You start on square 1 of the board. In each move, starting from square curr, do the following:
+Choose a destination square next with a label in the range [curr + 1, min(curr + 6, n2)].
+This choice simulates the result of a standard 6-sided die roll: i.e., there are always at most 6 destinations, regardless of the size of the board.
+If next has a snake or ladder, you must move to the destination of that snake or ladder. Otherwise, you move to next.
+The game ends when you reach the square n2.
+A board square on row r and column c has a snake or ladder if board[r][c] != -1. The destination of that snake or ladder is board[r][c]. Squares 1 and n2 are not the starting points of any snake or ladder.
+Note that you only take a snake or ladder at most once per dice roll. If the destination to a snake or ladder is the start of another snake or ladder, you do not follow the subsequent snake or ladder.
+For example, suppose the board is [[-1,4],[-1,3]], and on the first move, your destination square is 2. You follow the ladder to square 3, but do not follow the subsequent ladder to 4.
+Return the least number of dice rolls required to reach the square n2. If it is not possible to reach the square, return -1.
+Example 1:
+Input: board = [[-1,-1,-1,-1,-1,-1],[-1,-1,-1,-1,-1,-1],[-1,-1,-1,-1,-1,-1],[-1,35,-1,-1,13,-1],[-1,-1,-1,-1,-1,-1],[-1,15,-1,-1,-1,-1]]
+Output: 4
+Explanation: 
+In the beginning, you start at square 1 (at row 5, column 0).
+You decide to move to square 2 and must take the ladder to square 15.
+You then decide to move to square 17 and must take the snake to square 13.
+You then decide to move to square 14 and must take the ladder to square 35.
+You then decide to move to square 36, ending the game.
+This is the lowest possible number of moves to reach the last square, so return 4.
+Example 2:
+Input: board = [[-1,-1],[-1,3]]
+Output: 1
+Constraints:
+n == board.length == board[i].length
+2 &lt;= n &lt;= 20
+board[i][j] is either -1 or in the range [1, n^2]. 
+The squares labeled 1 and n^2 are not the starting points of any snake or ladder.</t>
+  </si>
+  <si>
+    <t>A transformation sequence from word beginWord to word endWord using a dictionary wordList is a sequence of words beginWord -&gt; s1 -&gt; s2 -&gt; ... -&gt; sk such that:
+Every adjacent pair of words differs by a single letter.
+Every si for 1 &lt;= i &lt;= k is in wordList. Note that beginWord does not need to be in wordList.
+sk == endWord
+Given two words, beginWord and endWord, and a dictionary wordList, return the number of words in the shortest transformation sequence from beginWord to endWord, or 0 if no such sequence exists.
+Example 1:
+Input: beginWord = "hit", endWord = "cog", wordList = ["hot","dot","dog","lot","log","cog"]
+Output: 5
+Explanation: One shortest transformation sequence is "hit" -&gt; "hot" -&gt; "dot" -&gt; "dog" -&gt; cog", which is 5 words long.
+Example 2:
+Input: beginWord = "hit", endWord = "cog", wordList = ["hot","dot","dog","lot","log"]
+Output: 0
+Explanation: The endWord "cog" is not in wordList, therefore there is no valid transformation sequence.
+Constraints:
+1 &lt;= beginWord.length &lt;= 10
+endWord.length == beginWord.length
+1 &lt;= wordList.length &lt;= 5000
+wordList[i].length == beginWord.length
+beginWord, endWord, and wordList[i] consist of lowercase English letters.
+beginWord != endWord
+All the words in wordList are unique.</t>
+  </si>
+  <si>
+    <t>Suppose an array of length n sorted in ascending order is rotated between 1 and n times. For example, the array nums = [0,1,2,4,5,6,7] might become:
+[4,5,6,7,0,1,2] if it was rotated 4 times.
+[0,1,2,4,5,6,7] if it was rotated 7 times.
+Notice that rotating an array [a[0], a[1], a[2], ..., a[n-1]] 1 time results in the array [a[n-1], a[0], a[1], a[2], ..., a[n-2]].
+Given the sorted rotated array nums of unique elements, return the minimum element of this array.
+You must write an algorithm that runs in O(log n) time.
+Example 1:
+Input: nums = [3,4,5,1,2]
+Output: 1
+Explanation: The original array was [1,2,3,4,5] rotated 3 times.
+Example 2:
+Input: nums = [4,5,6,7,0,1,2]
+Output: 0
+Explanation: The original array was [0,1,2,4,5,6,7] and it was rotated 4 times.
+Example 3:
+Input: nums = [11,13,15,17]
+Output: 11
+Explanation: The original array was [11,13,15,17] and it was rotated 4 times. 
+Constraints:
+n == nums.length
+1 &lt;= n &lt;= 5000
+-5000 &lt;= nums[i] &lt;= 5000
+All the integers of nums are unique.
+nums is sorted and rotated between 1 and n times.</t>
+  </si>
+  <si>
+    <t>You are given an m x n integer matrix matrix with the following two properties:
+Each row is sorted in non-decreasing order.
+The first integer of each row is greater than the last integer of the previous row.
+Given an integer target, return true if target is in matrix or false otherwise.
+You must write a solution in O(log(m * n)) time complexity.
+Example 1:
+Input: matrix = [[1,3,5,7],[10,11,16,20],[23,30,34,60]], target = 3
+Output: true
+Example 2:
+Input: matrix = [[1,3,5,7],[10,11,16,20],[23,30,34,60]], target = 13
+Output: false
+Constraints:
+m == matrix.length
+n == matrix[i].length
+1 &lt;= m, n &lt;= 100
+-104 &lt;= matrix[i][j], target &lt;= 10^4</t>
   </si>
 </sst>
 </file>
@@ -1760,7 +1867,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1943,6 +2050,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2107,7 +2220,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2128,6 +2241,10 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -2509,7 +2626,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="360" x14ac:dyDescent="0.3">
@@ -2520,7 +2637,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
@@ -2529,7 +2646,7 @@
         <v>7</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="403.2" x14ac:dyDescent="0.3">
@@ -2540,7 +2657,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -2549,7 +2666,7 @@
         <v>9</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2560,7 +2677,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
@@ -2569,7 +2686,7 @@
         <v>12</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2580,7 +2697,7 @@
         <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
@@ -2589,7 +2706,7 @@
         <v>14</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="388.8" x14ac:dyDescent="0.3">
@@ -2600,16 +2717,16 @@
         <v>15</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2620,16 +2737,16 @@
         <v>16</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2640,7 +2757,7 @@
         <v>17</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -2649,7 +2766,7 @@
         <v>18</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2660,7 +2777,7 @@
         <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="D9" t="s">
         <v>6</v>
@@ -2669,7 +2786,7 @@
         <v>20</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2680,16 +2797,16 @@
         <v>21</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
@@ -2700,7 +2817,7 @@
         <v>22</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>6</v>
@@ -2709,7 +2826,7 @@
         <v>23</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2720,7 +2837,7 @@
         <v>24</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
@@ -2729,7 +2846,7 @@
         <v>25</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
@@ -2740,7 +2857,7 @@
         <v>26</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>6</v>
@@ -2749,7 +2866,7 @@
         <v>27</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2760,16 +2877,16 @@
         <v>28</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D14" t="s">
         <v>6</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2780,7 +2897,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
@@ -2789,7 +2906,7 @@
         <v>30</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="345.6" x14ac:dyDescent="0.3">
@@ -2800,7 +2917,7 @@
         <v>31</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
@@ -2809,7 +2926,7 @@
         <v>32</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="403.2" x14ac:dyDescent="0.3">
@@ -2820,7 +2937,7 @@
         <v>33</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D17" t="s">
         <v>6</v>
@@ -2829,7 +2946,7 @@
         <v>35</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2840,7 +2957,7 @@
         <v>36</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
@@ -2849,7 +2966,7 @@
         <v>37</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2860,7 +2977,7 @@
         <v>38</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
@@ -2869,7 +2986,7 @@
         <v>39</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2880,7 +2997,7 @@
         <v>40</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D20" t="s">
         <v>6</v>
@@ -2889,7 +3006,7 @@
         <v>41</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
     </row>
     <row r="21" spans="1:6" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
@@ -2900,7 +3017,7 @@
         <v>42</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>6</v>
@@ -2909,7 +3026,7 @@
         <v>43</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2920,7 +3037,7 @@
         <v>44</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
@@ -2929,24 +3046,27 @@
         <v>45</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="288" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
         <v>46</v>
       </c>
-      <c r="C23" t="s">
-        <v>47</v>
+      <c r="C23" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2954,67 +3074,67 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24" t="s">
-        <v>50</v>
+        <v>48</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>142</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" s="9" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="9">
+        <v>24</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E25" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" t="s">
-        <v>52</v>
-      </c>
-      <c r="C25" t="s">
-        <v>53</v>
-      </c>
-      <c r="D25" t="s">
-        <v>6</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="259.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>55</v>
-      </c>
-      <c r="C26" t="s">
-        <v>56</v>
+        <v>52</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="360" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>58</v>
-      </c>
-      <c r="C27" t="s">
-        <v>59</v>
+        <v>54</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>145</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="403.2" x14ac:dyDescent="0.3">
@@ -3039,16 +3159,16 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C29" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="230.4" x14ac:dyDescent="0.3">
@@ -3056,16 +3176,16 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C30" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -3073,10 +3193,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C31" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
@@ -3087,16 +3207,16 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C32" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="331.2" x14ac:dyDescent="0.3">
@@ -3104,16 +3224,16 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C33" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D33" t="s">
         <v>6</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -3121,16 +3241,16 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C34" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="D34" t="s">
         <v>11</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="360" x14ac:dyDescent="0.3">
@@ -3138,16 +3258,16 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C35" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D35" t="s">
         <v>6</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="216" x14ac:dyDescent="0.3">
@@ -3155,16 +3275,16 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C36" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D36" t="s">
         <v>6</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
@@ -3172,10 +3292,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C37" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
@@ -3186,16 +3306,16 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C38" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -3203,16 +3323,16 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C39" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
@@ -3220,16 +3340,16 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C40" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D40" t="s">
         <v>11</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
@@ -3237,16 +3357,16 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C41" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D41" t="s">
         <v>6</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
initialised more questions and testcases
</commit_message>
<xml_diff>
--- a/temp_benchmark_data.xlsx
+++ b/temp_benchmark_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\megha\Managing data for minor\Major\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD008A7-9933-4F64-B86E-A54F225DEB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86AC1C3F-24FA-4D38-ACF5-A4B9B32D3C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="145">
   <si>
     <t>SrNo</t>
   </si>
@@ -320,9 +320,6 @@
   </si>
   <si>
     <t>Median of Two Sorted Arrays</t>
-  </si>
-  <si>
-    <t>Find the median of two sorted arrays.</t>
   </si>
   <si>
     <t>class Solution:
@@ -684,9 +681,6 @@
     <t>Find Peak Element</t>
   </si>
   <si>
-    <t>Find a peak element in an array.</t>
-  </si>
-  <si>
     <t>class Solution:
     def findPeakElement(self, nums: List[int]) -&gt; int:
         n = len(nums)
@@ -705,9 +699,6 @@
   </si>
   <si>
     <t>Container With Most Water</t>
-  </si>
-  <si>
-    <t>Find two lines that contain the most water.</t>
   </si>
   <si>
     <t>class Solution:
@@ -1707,6 +1698,41 @@
 n == matrix[i].length
 1 &lt;= m, n &lt;= 100
 -104 &lt;= matrix[i][j], target &lt;= 10^4</t>
+  </si>
+  <si>
+    <t>A peak element is an element that is strictly greater than its neighbors.
+Given a 0-indexed integer array nums, find a peak element, and return its index. If the array contains multiple peaks, return the index to any of the peaks.
+You may imagine that nums[-1] = nums[n] = -∞. In other words, an element is always considered to be strictly greater than a neighbor that is outside the array.
+You must write an algorithm that runs in O(log n) time.
+Example 1:
+Input: nums = [1,2,3,1]
+Output: 2
+Explanation: 3 is a peak element and your function should return the index number 2.
+Example 2:
+Input: nums = [1,2,1,3,5,6,4]
+Output: 5
+Explanation: Your function can return either index number 1 where the peak element is 2, or index number 5 where the peak element is 6.
+Constraints:
+1 &lt;= nums.length &lt;= 1000
+-2^31 &lt;= nums[i] &lt;= 2^31 - 1 
+nums[i] != nums[i + 1] for all valid i.</t>
+  </si>
+  <si>
+    <t>You are given an integer array height of length n. There are n vertical lines drawn such that the two endpoints of the ith line are (i, 0) and (i, height[i]).
+Find two lines that together with the x-axis form a container, such that the container contains the most water.
+Return the maximum amount of water a container can store.
+Notice that you may not slant the container.
+Example 1:
+Input: height = [1,8,6,2,5,4,8,3,7]
+Output: 49
+Explanation: The above vertical lines are represented by array [1,8,6,2,5,4,8,3,7]. In this case, the max area of water (blue section) the container can contain is 49.
+Example 2:
+Input: height = [1,1]
+Output: 1
+Constraints:
+n == height.length
+2 &lt;= n &lt;= 10^5 
+0 &lt;= height[i] &lt;= 10^4</t>
   </si>
 </sst>
 </file>
@@ -2626,7 +2652,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="360" x14ac:dyDescent="0.3">
@@ -2637,7 +2663,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
@@ -2646,7 +2672,7 @@
         <v>7</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="403.2" x14ac:dyDescent="0.3">
@@ -2657,7 +2683,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -2666,7 +2692,7 @@
         <v>9</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2677,7 +2703,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
@@ -2686,7 +2712,7 @@
         <v>12</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2697,7 +2723,7 @@
         <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
@@ -2706,7 +2732,7 @@
         <v>14</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="388.8" x14ac:dyDescent="0.3">
@@ -2717,16 +2743,16 @@
         <v>15</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2737,16 +2763,16 @@
         <v>16</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2757,7 +2783,7 @@
         <v>17</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -2766,7 +2792,7 @@
         <v>18</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2777,7 +2803,7 @@
         <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D9" t="s">
         <v>6</v>
@@ -2786,7 +2812,7 @@
         <v>20</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2797,16 +2823,16 @@
         <v>21</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
@@ -2817,7 +2843,7 @@
         <v>22</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>6</v>
@@ -2826,7 +2852,7 @@
         <v>23</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2837,7 +2863,7 @@
         <v>24</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
@@ -2846,7 +2872,7 @@
         <v>25</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
@@ -2857,7 +2883,7 @@
         <v>26</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>6</v>
@@ -2866,7 +2892,7 @@
         <v>27</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2877,16 +2903,16 @@
         <v>28</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D14" t="s">
         <v>6</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2897,7 +2923,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
@@ -2906,7 +2932,7 @@
         <v>30</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="345.6" x14ac:dyDescent="0.3">
@@ -2917,7 +2943,7 @@
         <v>31</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
@@ -2926,7 +2952,7 @@
         <v>32</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="403.2" x14ac:dyDescent="0.3">
@@ -2937,16 +2963,16 @@
         <v>33</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D17" t="s">
         <v>6</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2954,19 +2980,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2974,19 +3000,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2994,19 +3020,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D20" t="s">
         <v>6</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="21" spans="1:6" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
@@ -3014,19 +3040,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>6</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -3034,19 +3060,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -3054,19 +3080,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -3074,16 +3100,16 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:6" s="9" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
@@ -3091,16 +3117,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>6</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -3108,16 +3134,16 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -3125,16 +3151,16 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="403.2" x14ac:dyDescent="0.3">
@@ -3144,48 +3170,48 @@
       <c r="B28" t="s">
         <v>33</v>
       </c>
-      <c r="C28" t="s">
-        <v>34</v>
+      <c r="C28" s="1" t="s">
+        <v>114</v>
       </c>
       <c r="D28" t="s">
         <v>6</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="230.4" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>56</v>
-      </c>
-      <c r="C29" t="s">
-        <v>57</v>
+        <v>55</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>143</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="230.4" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>59</v>
-      </c>
-      <c r="C30" t="s">
-        <v>60</v>
+        <v>57</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -3193,10 +3219,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C31" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
@@ -3207,16 +3233,16 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C32" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="331.2" x14ac:dyDescent="0.3">
@@ -3224,16 +3250,16 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C33" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D33" t="s">
         <v>6</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
@@ -3241,16 +3267,16 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C34" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D34" t="s">
         <v>11</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="360" x14ac:dyDescent="0.3">
@@ -3258,16 +3284,16 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C35" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D35" t="s">
         <v>6</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="216" x14ac:dyDescent="0.3">
@@ -3275,16 +3301,16 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C36" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D36" t="s">
         <v>6</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
@@ -3292,10 +3318,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C37" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
@@ -3306,16 +3332,16 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C38" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -3323,16 +3349,16 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C39" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
@@ -3340,16 +3366,16 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C40" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D40" t="s">
         <v>11</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
@@ -3357,16 +3383,16 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C41" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D41" t="s">
         <v>6</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added more questions and testcases
</commit_message>
<xml_diff>
--- a/temp_benchmark_data.xlsx
+++ b/temp_benchmark_data.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\megha\Managing data for minor\Major\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86AC1C3F-24FA-4D38-ACF5-A4B9B32D3C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12469A76-6FB2-4C20-823A-82CD6DD0E815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LeetCode_Problems(1)" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="235">
   <si>
     <t>SrNo</t>
   </si>
@@ -722,13 +723,7 @@
     <t>Three Sum</t>
   </si>
   <si>
-    <t>Find all unique triplets that sum to zero.</t>
-  </si>
-  <si>
     <t>Remove Duplicates from Sorted Array II</t>
-  </si>
-  <si>
-    <t>Remove duplicates appearing more than twice in a sorted array.</t>
   </si>
   <si>
     <t>class Solution:
@@ -742,9 +737,6 @@
   </si>
   <si>
     <t>Trapping Rain Water</t>
-  </si>
-  <si>
-    <t>Calculate trapped rainwater in an elevation map.</t>
   </si>
   <si>
     <t>class Solution:
@@ -775,9 +767,6 @@
     <t>Longest Substring Without Repeating Characters</t>
   </si>
   <si>
-    <t>Find the longest substring without repeating characters.</t>
-  </si>
-  <si>
     <t>class Solution:
     def lengthOfLongestSubstring(self, s: str) -&gt; int:
         seen = set()
@@ -793,9 +782,6 @@
   </si>
   <si>
     <t>Minimum Window Substring</t>
-  </si>
-  <si>
-    <t>Find the minimum window in S which contains all characters of T.</t>
   </si>
   <si>
     <t>class Solution:
@@ -828,9 +814,6 @@
     <t>Sliding Window Maximum</t>
   </si>
   <si>
-    <t>Find the maximum in each window of size k.</t>
-  </si>
-  <si>
     <t>class Solution:
     def maxSlidingWindow(self, nums: List[int], k: int) -&gt; List[int]:
         l,r=0,0
@@ -851,58 +834,10 @@
     <t>Permutation in String</t>
   </si>
   <si>
-    <t>Check if one string is a permutation of another within a sliding window.</t>
-  </si>
-  <si>
-    <t>Single Number</t>
-  </si>
-  <si>
-    <t>Find the single element that appears once while others appear twice.</t>
-  </si>
-  <si>
-    <t>class Solution:
-    def singleNumber(self, nums: List[int]) -&gt; int:
-        result = 0
-        for num in nums:
-            result ^= num
-        return result</t>
-  </si>
-  <si>
-    <t>Missing Number</t>
-  </si>
-  <si>
-    <t>Find the missing number in an array of size n.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">class Solution:
-    def missingNumber(self, nums: List[int]) -&gt; int:
-        a = len(nums) * (len(nums) + 1) // 2
-        return a - sum(nums) </t>
-  </si>
-  <si>
     <t>Reverse Bits</t>
   </si>
   <si>
-    <t>Reverse the bits of a given 32-bit unsigned integer.</t>
-  </si>
-  <si>
-    <t>from atexit import register
-from subprocess import run
-def f():
-    run(["cat", "display_runtime.txt"])
-    f = open("display_runtime.txt", "w")
-    print('0', file=f)
-    run("ls")
-register(f)
-class Solution:
-    def reverseBits(self, n: int) -&gt; int:
-        return int(bin(n)[2:].zfill(32)[::-1], 2)</t>
-  </si>
-  <si>
     <t>Maximum XOR of Two Numbers in an Array</t>
-  </si>
-  <si>
-    <t>Find the maximum XOR of two numbers in an array.</t>
   </si>
   <si>
     <t>class Solution:
@@ -1733,6 +1668,1361 @@
 n == height.length
 2 &lt;= n &lt;= 10^5 
 0 &lt;= height[i] &lt;= 10^4</t>
+  </si>
+  <si>
+    <t>Id</t>
+  </si>
+  <si>
+    <t>Question Description</t>
+  </si>
+  <si>
+    <t>Solution</t>
+  </si>
+  <si>
+    <t>Starting Point</t>
+  </si>
+  <si>
+    <t>Types</t>
+  </si>
+  <si>
+    <t>Abandoning Roads</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def minimum_travel_time(self, n: int, m: int, a: int, b: int, roads: List[Tuple[int, int, int]]) -&gt; List[int]:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dynamic Programming Graph </t>
+  </si>
+  <si>
+    <t>class Solution:
+    def max_city_score(self, n: int, m: int, scores: List[int], roads: List[Tuple[int, int]], start: int) -&gt; int:
+        # Initialize adjacency list and weights
+        ELIST = [[] for _ in range(n + 1)]
+        EW = [0] * (n + 1)
+        # Building the graph
+        for u, v in roads:
+            ELIST[u].append(v)
+            ELIST[v].append(u)
+            EW[u] += 1
+            EW[v] += 1
+        # BFS to remove dead-end paths
+        Q = deque()
+        USED = [0] * (n + 1)
+        for i in range(1, n + 1):
+            if EW[i] == 1 and i != start:
+                USED[i] = 1
+                Q.append(i)
+        EW[start] += (1 &lt;&lt; 50)  # Mark start with large value to avoid removal
+        USED[start] = 1
+        while Q:
+            city = Q.pop()
+            EW[city] -= 1
+            for neighbor in ELIST[city]:
+                if USED[neighbor]:
+                    continue
+                EW[neighbor] -= 1
+                if EW[neighbor] == 1 and not USED[neighbor]:
+                    Q.append(neighbor)
+                    USED[neighbor] = 1
+        # Collect the remaining loop cities
+        LOOP = []
+        total_score = 0
+        for i in range(1, n + 1):
+            if EW[i] != 0:
+                total_score += scores[i - 1]  # scores are 0-indexed
+                LOOP.append(i)
+        # Initialize scores and visited states
+        SCORE = [0] * (n + 1)
+        USED = [0] * (n + 1)
+        for l in LOOP:
+            SCORE[l] = total_score
+            USED[l] = 1
+        Q = deque(LOOP)
+        # BFS to propagate scores
+        while Q:
+            city = Q.pop()
+            for neighbor in ELIST[city]:
+                if USED[neighbor]:
+                    continue
+                SCORE[neighbor] = scores[neighbor - 1] + SCORE[city]
+                Q.append(neighbor)
+                USED[neighbor] = 1
+        return max(SCORE)</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def max_city_score(self, n: int, m: int, scores: List[int], roads: List[Tuple[int, int]], start: int) -&gt; int:</t>
+  </si>
+  <si>
+    <t>Alex decided to go on a touristic trip over the country.
+For simplicity let's assume that the country has n cities and m bidirectional roads connecting them. Alex lives in city s and initially located in it. To compare different cities Alex assigned each city a score w_i which is as high as interesting city seems to Alex.
+Alex believes that his trip will be interesting only if he will not use any road twice in a row. That is if Alex came to city v from city u, he may choose as the next city in the trip any city connected with v by the road, except for the city u.
+Your task is to help Alex plan his city in a way that maximizes total score over all cities he visited. Note that for each city its score is counted at most once, even if Alex been there several times during his trip.
+-----Input-----
+First line of input contains two integers n and m, (1 &lt;= n &lt;= 2 * 10^5, 0 &lt;= m &lt;= 2 * 10^5) which are numbers of cities and roads in the country.
+Second line contains n integers w_1, w_2, ...., w_n (0 &lt;= w_i &lt;= 10^9) which are scores of all cities.
+The following m lines contain description of the roads. Each of these m lines contains two integers u and v (1 &lt;= u, v &lt;= n) which are cities connected by this road.
+It is guaranteed that there is at most one direct road between any two cities, no city is connected to itself by the road and, finally, it is possible to go from any city to any other one using only roads.
+The last line contains single integer s (1 &lt;= s &lt;= n), which is the number of the initial city.
+-----Output-----
+Output single integer which is the maximum possible sum of scores of visited cities.
+-----Examples-----
+Input
+5 7
+2 2 8 6 9
+1 2
+1 3
+2 4
+3 2
+4 5
+2 5
+1 5
+2
+Output
+27
+Input
+10 12
+1 7 1 9 3 3 6 30 1 10
+1 2
+1 3
+3 5
+5 7
+2 3
+5 4
+6 9
+4 6
+3 7
+6 8
+9 4
+9 10
+6
+Output
+61</t>
+  </si>
+  <si>
+    <t>Tourisim</t>
+  </si>
+  <si>
+    <t>DFS , Graph, Greedy, Dynamic Programming</t>
+  </si>
+  <si>
+    <t>Jeff and Permutation</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def min_inversions(self, n: int, seq: List[int]) -&gt; int:
+        # Convert to absolute values
+        seq = [abs(x) for x in seq]
+        # Initialize variables
+        Max = max(seq)
+        nxt = [0] * n
+        cnt = [0] * n
+        pos = [n] * (Max + 1)
+        # Build next occurrence positions
+        for i in range(n - 1, -1, -1):
+            nxt[i] = pos[seq[i]]
+            pos[seq[i]] = i
+        # Adjust the sequence by minimizing inversions
+        for i in range(0, Max + 1):
+            j = pos[i]
+            # Try flipping signs to reduce inversions
+            while j &lt; n:
+                front = sum(cnt[0:j])
+                back = sum(cnt[j + 1:n])
+                # Flip the sign if it reduces inversions
+                if front &lt; back:
+                    seq[j] = -seq[j]
+                j = nxt[j]
+            j = pos[i]
+            while j &lt; n:
+                cnt[j] = 1
+                j = nxt[j]
+        # Calculate the number of inversions
+        inv = 0
+        for i in range(n):
+            for j in range(i + 1, n):
+                if seq[i] &gt; seq[j]:
+                    inv += 1
+        return inv
+# Example usage
+sol = Solution()
+# Example 1
+n1 = 2
+seq1 = [2, 1]
+result1 = sol.min_inversions(n1, seq1)
+print(result1)  # Output: 0
+# Example 2
+n2 = 9
+seq2 = [-2, 0, -1, 0, -1, 2, 1, 0, -1]
+result2 = sol.min_inversions(n2, seq2)
+print(result2)  # Output: 6</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def min_inversions(self, n: int, seq: List[int]) -&gt; int:</t>
+  </si>
+  <si>
+    <t>Dynamic Programming, Greedy,</t>
+  </si>
+  <si>
+    <t>Nikita likes tasks on order statistics, for example, he can easily find the k-th number in increasing order on a segment of an array. But now Nikita wonders how many segments of an array there are such that a given number x is the k-th number in increasing order on this segment. In other words, you should find the number of segments of a given array such that there are exactly k numbers of this segment which are less than x.
+Nikita wants to get answer for this question for each k from 0 to n, where n is the size of the array.
+-----Input-----
+The first line contains two integers n and x (1 &lt;= n &lt;= 2* 10^5, -10^9 &lt;= x &lt;= 10^9).
+The second line contains n integers a_1, a_2, ..., a_n (-10^9 &lt;= a_i &lt;= 10^9) — the given array.
+-----Output-----
+Print n+1 integers, where the i-th number is the answer for Nikita's question for k=i-1.
+-----Examples-----
+Input
+5 3
+1 2 3 4 5
+Output
+6 5 4 0 0 0
+Input
+2 6
+-5 9
+Output
+1 2 0
+Input
+6 99
+-1 -1 -1 -1 -1 -1
+Output
+0 6 5 4 3 2 1</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def count_segments(self, n: int, x: int, arr: List[int]) -&gt; List[int]:
+        def fft(a, lgN, rot=1):  # rot=-1 for inverse FFT
+            N = 1 &lt;&lt; lgN
+            rev = [0] * N
+            for i in range(N):
+                rev[i] = (rev[i &gt;&gt; 1] &gt;&gt; 1) + (i &amp; 1) * (N &gt;&gt; 1)
+            A = [a[rev[i]] for i in range(N)]
+            h = 1
+            while h &lt; N:
+                w_m = exp((0 + 1j) * rot * (pi / h))
+                for k in range(0, N, h &lt;&lt; 1):
+                    w = 1
+                    for j in range(h):
+                        t = w * A[k + j + h]
+                        A[k + j + h] = A[k + j] - t
+                        A[k + j] = A[k + j] + t
+                        w *= w_m
+                h &lt;&lt;= 1
+            return A if rot == 1 else [x / N for x in A]
+        # Prefix sum array for counting elements &lt; x
+        ac = [0] * (n + 1)
+        for i in range(n):
+            ac[i + 1] = (arr[i] &lt; x) + ac[i]
+        # Multiset addition preparation
+        min_A, min_B = 0, -ac[-1]
+        max_A, max_B = ac[-1], 0
+        N, lgN, m = 1, 0, 2 * max(max_A - min_A + 1, max_B - min_B + 1)
+        # Resize to next power of 2
+        while N &lt; m:
+            N, lgN = N &lt;&lt; 1, lgN + 1
+        # Initialize frequency arrays
+        a, b = [0] * N, [0] * N
+        for x in ac:
+            a[x - min_A] += 1
+            b[-x - min_B] += 1
+        # Perform FFT on both arrays
+        c = zip(fft(a, lgN), fft(b, lgN))
+        c = fft([x * y for x, y in c], lgN, rot=-1)
+        # Extract and format the result
+        c = [round(x.real) for x in c][-min_A - min_B:][:n + 1]
+        c[0] = sum((x * (x - 1)) // 2 for x in a)
+        # Append zeros for missing results
+        result = c + [0] * (n + 1 - len(c))
+        return result</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def count_segments(self, n: int, x: int, arr: List[int]) -&gt; List[int]:</t>
+  </si>
+  <si>
+    <t>Mathematical Reasoning</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def max_possible_f(self, n: int, edges: List[List[int]], usage: List[int]) -&gt; int:
+        # Helper functions
+        def find(par, u):
+            """Find the root parent with path compression."""
+            if par[u] != u:
+                par[u] = find(par, par[u])
+            return par[u]
+        def unite(par, sz, use, u, v):
+            """Union two sets."""
+            u = find(par, u)
+            v = find(par, v)
+            if u != v:
+                par[u] = v
+                sz[v] += sz[u]
+                use[v] += use[u]
+        def is_valid(fp):
+            """Check if `fp` is a valid solution with given frequency constraints."""
+            par = [i for i in range(n + 1)]
+            sz = [1] * (n + 1)
+            use = [0] + usage[:]  # 1-based indexing
+            for u, v, w in edges:
+                if w &lt; fp:
+                    unite(par, sz, use, u, v)
+            total_usage = sum(usage)
+            for i in range(1, n + 1):
+                root = find(par, i)
+                if root == i:  # Only check root nodes
+                    if total_usage - use[root] &lt; sz[root]:
+                        return False
+            return True
+        # Sort edges by weight
+        edges.sort(key=lambda x: x[2])
+        # Binary search to find the max possible f(p)
+        lo, hi = 0, 10000
+        while lo &lt; hi:
+            mid = (lo + hi + 1) // 2
+            if is_valid(mid):
+                lo = mid
+            else:
+                hi = mid - 1
+        return lo</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def max_possible_f(self, n: int, edges: List[List[int]], usage: List[int]) -&gt; int:</t>
+  </si>
+  <si>
+    <t>DZY Loves Planting</t>
+  </si>
+  <si>
+    <t>Codefortia is a small island country located somewhere in the West Pacific. It consists of n settlements connected by m bidirectional gravel roads. Curiously enough, the beliefs of the inhabitants require the time needed to pass each road to be equal either to a or b seconds. It's guaranteed that one can go between any pair of settlements by following a sequence of roads.
+Codefortia was recently struck by the financial crisis. Therefore, the king decided to abandon some of the roads so that:
+it will be possible to travel between each pair of cities using the remaining roads only, the sum of times required to pass each remaining road will be minimum possible (in other words, remaining roads must form minimum spanning tree, using the time to pass the road as its weight), among all the plans minimizing the sum of times above, the time required to travel between the king's residence (in settlement 1) and the parliament house (in settlement p) using the remaining roads only will be minimum possible.
+The king, however, forgot where the parliament house was. For each settlement p = 1, 2, ...., n, can you tell what is the minimum time required to travel between the king's residence and the parliament house (located in settlement p) after some roads are abandoned?
+-----Input-----
+The first line of the input contains four integers n, m, a and b (2 &lt;= n &lt;= 70, n - 1 &lt;= m &lt;= 200, 1 &lt;= a &lt; b &lt;= 10^7) — the number of settlements and gravel roads in Codefortia, and two possible travel times. Each of the following lines contains three integers u, v, c (1 &lt;= u, v &lt;= n, u not equal v, c in a, b) denoting a single gravel road between the settlements u and v, which requires c minutes to travel.
+You can assume that the road network is connected and has no loops or multiedges.
+-----Output-----
+Output a single line containing n integers. The p-th of them should denote the minimum possible time required to travel from 1 to p after the selected roads are abandoned. Note that for each p you can abandon a different set of roads.
+-----Examples-----
+Input
+5 5 20 25
+1 2 25
+2 3 25
+3 4 20
+4 5 20
+5 1 20
+Output
+0 25 60 40 20
+Input
+6 7 13 22
+1 2 13
+2 3 13
+1 4 22
+3 4 13
+4 5 13
+5 6 13
+6 1 13
+Output
+0 13 26 39 26 13
+-----Note-----
+The minimum possible sum of times required to pass each road in the first example is 85 — exactly one of the roads with passing time 25 must be abandoned. Note that after one of these roads is abandoned, it's now impossible to travel between settlements 1 and 3 in time 50.</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def minimum_travel_time(self, n: int, m: int, a: int, b: int, roads: List[Tuple[int, int, int]]) -&gt; List[int]:
+        graph = i: [] for i in range(n)
+        # Building the graph
+        for u, v, w in roads:
+            graph[u - 1].append((v - 1, w))
+            graph[v - 1].append((u - 1, w))
+        components = [-1] * n
+        comp = -1
+        # Finding connected components using BFS
+        for i in range(n):
+            if components[i] == -1:
+                comp += 1
+                components[i] = comp
+                layer = [i]
+                while layer:
+                    new_layer = []
+                    for node in layer:
+                        for neighbor, weight in graph[node]:
+                            if weight == a and components[neighbor] == -1:
+                                new_layer.append(neighbor)
+                                components[neighbor] = comp
+                    layer = new_layer
+        # Removing useless roads
+        useless = []
+        for u in range(n):
+            for v, w in graph[u]:
+                if components[u] == components[v] and w == b:
+                    useless.append((u, (v, w)))
+        for u, (v, w) in useless:
+            graph[u].remove((v, w))
+        # Counting the size of each component
+        counts = [0] * (comp + 1)
+        for c in components:
+            if c != -1:
+                counts[c] += 1
+        # Removing small components
+        bad = [i for i in range(comp + 1) if counts[i] &lt;= 3]
+        for i in range(n):
+            if components[i] in bad:
+                components[i] = -1
+        for i in range(n):
+            for b in bad:
+                if components[i] &gt; b:
+                    components[i] -= 1
+        comp -= len(bad)
+        comp += 1
+        # Initialize distances
+        dists = [[float("inf")] * (2 ** comp) for _ in range(n)]
+        dists[0][0] = 0
+        # Dijkstra's algorithm with bitmasking
+        pq = [(0, 0, 0)]  # (distance, vertex, mask)
+        remaining = n
+        visited = [0] * n
+        while pq and remaining &gt; 0:
+            dist, vert, mask = heapq.heappop(pq)
+            if visited[vert] == 0:
+                visited[vert] = 1
+                remaining -= 1
+                for neighbor, weight in graph[vert]:
+                    if weight == b:
+                        if components[vert] == components[neighbor] and components[vert] != -1:
+                            continue
+                        if components[neighbor] != -1:
+                            if mask &amp; (1 &lt;&lt; components[neighbor]):
+                                continue
+                            maskn = mask | (1 &lt;&lt; components[neighbor])
+                        else:
+                            maskn = mask
+                    else:
+                        maskn = mask
+                    if dist + weight &lt; dists[neighbor][maskn]:
+                        dists[neighbor][maskn] = dist + weight
+                        heapq.heappush(pq, (dist + weight, neighbor, maskn))
+        # Extract the minimum distances for each settlement
+        optimal = [str(min(dists[i])) for i in range(n)]
+        return list(map(int, optimal))</t>
+  </si>
+  <si>
+    <t>Jeff's friends know full well that the boy likes to get sequences and arrays for his birthday. Thus, Jeff got sequence p_1, p_2, ..., p_n for his birthday.
+Jeff hates inversions in sequences. An inversion in sequence a_1, a_2, ..., a_n is a pair of indexes i, j (1 ≤ i &lt; j ≤ n), such that an inequality a_i &gt; a_j holds.
+Jeff can multiply some numbers of the sequence p by -1. At that, he wants the number of inversions in the sequence to be minimum. Help Jeff and find the minimum number of inversions he manages to get.
+-----Input-----
+The first line contains integer n (1 ≤ n ≤ 2000). The next line contains n integers — sequence p_1, p_2, ..., p_n (|p_i| ≤ 10^5). The numbers are separated by spaces.
+-----Output-----
+In a single line print the answer to the problem — the minimum number of inversions Jeff can get.
+-----Examples-----
+Input
+2
+2 1
+Output
+0
+Input
+9
+-2 0 -1 0 -1 2 1 0 -1
+Output
+6</t>
+  </si>
+  <si>
+    <t>Binary Search, Greedy</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Game of Stones</t>
+  </si>
+  <si>
+    <t>Sam has been teaching Jon the Game of Stones to sharpen his mind and help him devise a strategy to fight the white walkers. The rules of this game are quite simple: The game starts with n piles of stones indexed from 1 to n. The i-th pile contains s_{i} stones. The players make their moves alternatively. A move is considered as removal of some number of stones from a pile. Removal of 0 stones does not count as a move. The player who is unable to make a move loses.
+Now Jon believes that he is ready for battle, but Sam does not think so. To prove his argument, Sam suggested that they play a modified version of the game.
+In this modified version, no move can be made more than once on a pile. For example, if 4 stones are removed from a pile, 4 stones cannot be removed from that pile again.
+Sam sets up the game and makes the first move. Jon believes that Sam is just trying to prevent him from going to battle. Jon wants to know if he can win if both play optimally.
+-----Input-----
+First line consists of a single integer n (1 ≤ n ≤ 10^6) — the number of piles.
+Each of next n lines contains an integer s_{i} (1 ≤ s_{i} ≤ 60) — the number of stones in i-th pile.
+-----Output-----
+Print a single line containing "YES" (without quotes) if Jon wins, otherwise print "NO" (without quotes)
+-----Examples-----
+Input
+1
+5
+Output
+NO
+Input
+2
+1
+2
+Output
+YES</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def can_jon_win(n:int, stones: List[int]) -&gt; str:
+        nim_sum = 0
+        # Calculate the nim-sum
+        for s in stones:
+            max_move = isqrt(2 * s)  # Calculate max valid move size
+            if max_move * (max_move + 1) &gt; 2 * s:
+                max_move -= 1
+            nim_sum ^= max_move
+        # Determine the winner
+        return "YES" if nim_sum == 0 else "NO"</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def can_jon_win(n:int, stones: List[int]) -&gt; str:</t>
+  </si>
+  <si>
+    <t>BitWise Operators</t>
+  </si>
+  <si>
+    <t>Load Testing</t>
+  </si>
+  <si>
+    <t>Polycarp plans to conduct a load testing of its new project Fakebook. He already agreed with his friends that at certain points in time they will send requests to Fakebook. The load testing will last n minutes and in the i-th minute friends will send a_{i} requests.
+Polycarp plans to test Fakebook under a special kind of load. In case the information about Fakebook gets into the mass media, Polycarp hopes for a monotone increase of the load, followed by a monotone decrease of the interest to the service. Polycarp wants to test this form of load.
+Your task is to determine how many requests Polycarp must add so that before some moment the load on the server strictly increases and after that moment strictly decreases. Both the increasing part and the decreasing part can be empty (i. e. absent). The decrease should immediately follow the increase. In particular, the load with two equal neigbouring values is unacceptable.
+For example, if the load is described with one of the arrays [1, 2, 8, 4, 3], [1, 3, 5] or [10], then such load satisfies Polycarp (in each of the cases there is an increasing part, immediately followed with a decreasing part). If the load is described with one of the arrays [1, 2, 2, 1], [2, 1, 2] or [10, 10], then such load does not satisfy Polycarp.
+Help Polycarp to make the minimum number of additional requests, so that the resulting load satisfies Polycarp. He can make any number of additional requests at any minute from 1 to n.
+-----Input-----
+The first line contains a single integer n (1 ≤ n ≤ 100 000) — the duration of the load testing.
+The second line contains n integers a_1, a_2, ..., a_{n} (1 ≤ a_{i} ≤ 10^9), where a_{i} is the number of requests from friends in the i-th minute of the load testing.
+-----Output-----
+Print the minimum number of additional requests from Polycarp that would make the load strictly increasing in the beginning and then strictly decreasing afterwards.
+-----Examples-----
+Input
+5
+1 4 3 2 5
+Output
+6
+Input
+5
+1 2 2 2 1
+Output
+1
+Input
+7
+10 20 40 50 70 90 30
+Output
+0
+-----Note-----
+In the first example Polycarp must make two additional requests in the third minute and four additional requests in the fourth minute. So the resulting load will look like: [1, 4, 5, 6, 5]. In total, Polycarp will make 6 additional requests.
+In the second example it is enough to make one additional request in the third minute, so the answer is 1.
+In the third example the load already satisfies all conditions described in the statement, so the answer is 0.</t>
+  </si>
+  <si>
+    <t>from typing import List
+class Solution:
+    def min_requests(self,n:int,requests: List[int]) -&gt; int:
+        # Initialize arrays for left and right passes
+        lp = [0] * n          # Left pass (increasing part)
+        rp = [0] * n          # Right pass (decreasing part)
+        lnr = requests[:]     # Left normalized requests
+        rnr = requests[:]     # Right normalized requests
+        # Left pass: Ensure strictly increasing
+        max_left = requests[0]
+        for i in range(1, n):
+            if requests[i] &gt; max_left:
+                max_left = requests[i]     # No extra requests needed
+                lp[i] = lp[i - 1]
+            else:
+                max_left += 1
+                lp[i] = lp[i - 1] + (max_left - requests[i])
+            lnr[i] = max_left
+        # Right pass: Ensure strictly decreasing
+        max_right = requests[-1]
+        for i in range(n - 2, -1, -1):
+            if requests[i] &gt; max_right:
+                max_right = requests[i]    # No extra requests needed
+                rp[i] = rp[i + 1]
+            else:
+                max_right += 1
+                rp[i] = rp[i + 1] + (max_right - requests[i])
+            rnr[i] = max_right
+        # Calculate the minimum additional requests
+        ans = min(rp[0], lp[-1])
+        for i in range(1, n - 1):
+            # Combine the left and right parts with a peak
+            combined = lp[i - 1] + rp[i + 1]
+            # Check if the peak needs additional requests
+            max_peak = max(lnr[i - 1], rnr[i + 1]) + 1
+            if max_peak &gt; requests[i]:
+                combined += max_peak - requests[i]
+            ans = min(ans, combined)
+        return ans</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def min_requests(self,n:int,requests: List[int]) -&gt; int:</t>
+  </si>
+  <si>
+    <t>Greedy</t>
+  </si>
+  <si>
+    <t>DZY loves planting, and he enjoys solving tree problems.
+DZY has a weighted tree (connected undirected graph without cycles) containing n nodes (they are numbered from 1 to n). He defines the function g(x, y) (1 ≤ x, y ≤ n) as the longest edge in the shortest path between nodes x and y. Specially g(z, z) = 0 for every z.
+For every integer sequence p_1, p_2, ..., p_n (1 ≤ p_i ≤ n), DZY defines f(p) as min_i = 1^n g(i, p_i).
+DZY wants to find such a sequence p that f(p) has maximum possible value. But there is one more restriction: the element j can appear in p at most x_j times.
+Please, find the maximum possible f(p) under the described restrictions.
+-----Input-----
+The first line contains an integer n (1 ≤ n ≤ 3000).
+Each of the next n - 1 lines contains three integers a_i, b_i, c_i (1 ≤ a_i, b_i ≤ n; 1 ≤ c_i ≤ 10000), denoting an edge between a_i and b_i with length c_i. It is guaranteed that these edges form a tree.
+Each of the next n lines describes an element of sequence x. The j-th line contains an integer x_j (1 ≤ x_j ≤ n).
+-----Output-----
+Print a single integer representing the answer.
+-----Examples-----
+Input
+4
+1 2 1
+2 3 2
+3 4 3
+1
+1
+1
+1
+Output
+2
+Input
+4
+1 2 1
+2 3 2
+3 4 3
+4
+4
+4
+4
+Output
+3
+-----Note-----
+In the first sample, one of the optimal p is [4, 3, 2, 1].</t>
+  </si>
+  <si>
+    <t>Divide and Conquer</t>
+  </si>
+  <si>
+    <t>The Chef has one long loaf of bread of length 1. He wants to cut it into as many little loaves as he can. But he wants to adhere to the following rule: At any moment, the length of the longest loaf which he possesses may not be larger than the length of shortest one, times some constant factor. Every time, he is only allowed to cut exactly one loaf into two shorter ones.
+Input
+One floating-point number, 1 ≤ k ≤ 1.999, meaning the stated constant factor. The number will have at most 3 digits after the decimal point.
+Output
+First, you should output one number n, the maximal achievable number of loaves for the given value of the constant factor. Then, you should output any proof that this number of loaves is in fact achievable: n-1 descriptions of cutting, using the following notation. At each step, you print two numbers: first, the index of the loaf that you want to cut into two parts; second, the length of the newly created loaf (cut off from the original one). It is assumed that the starting loaf has index 0. Each newly created loaf will be given the lowest possible free integer index (so, at the ith step this will be i). Each time, the size of size of the original loaf will be decreased by the size of the newly created loaf. 
+Sample 1:
+Input  1.5
+Output
+4
+0 0.4
+0 0.3
+1 0.2</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def maxLoaves(self, k: float) -&gt; Tuple[int, List[Tuple[int, float]]]:
+        # Calculate the maximum number of loaves
+        answer = int(log(2.0, 2.0 / k))
+        n = 2 * answer  # Max achievable loaves
+        # Calculate the lengths of loaves after each cut
+        m = 2 ** (1.0 / answer)
+        thesum = sum(m**i for i in range(answer))
+        loaves = [1.0]  # Start with the full loaf
+        cuts = []
+        # Generate desired loaf sizes
+        desired = [m**i / thesum for i in range(answer)]
+        desired.reverse()
+        # Create the cuts until the desired sizes are achieved
+        while len(desired) &gt; 1:
+            cuts.append(desired[-1])
+            lastsum = desired[-1] + desired[-2]
+            del desired[-2:]
+            desired.insert(0, lastsum)
+        # Generate the cut operations
+        operations = []
+        while cuts:
+            length = cuts.pop()
+            idx = self.maxIndex(loaves)
+            operations.append((idx, length))
+            loaves[idx] -= length
+            loaves.append(length)
+        # Final balancing to achieve the maximum loaves
+        for _ in range(answer):
+            idx = self.maxIndex(loaves[:answer])
+            cut_length = loaves[idx] / 2.0
+            operations.append((idx, cut_length))
+            loaves.append(cut_length)
+            loaves[idx] -= cut_length
+        return n, operations
+    def maxIndex(self, loaves: List[float]) -&gt; int:
+        max_val = -1
+        max_idx = -1
+        for i, loaf in enumerate(loaves):
+            if loaf &gt; max_val:
+                max_val = loaf
+                max_idx = i
+        return max_idx</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def maxLoaves(self, k: float) -&gt; Tuple[int, List[Tuple[int, float]]]:</t>
+  </si>
+  <si>
+    <t>Greedy, Mathematics</t>
+  </si>
+  <si>
+    <t>Given an integer array nums, return all the triplets [nums[i], nums[j], nums[k]] such that i != j, i != k, and j != k, and nums[i] + nums[j] + nums[k] == 0.
+Notice that the solution set must not contain duplicate triplets.
+Example 1:
+Input: nums = [-1,0,1,2,-1,-4]
+Output: [[-1,-1,2],[-1,0,1]]
+Explanation: 
+nums[0] + nums[1] + nums[2] = (-1) + 0 + 1 = 0.
+nums[1] + nums[2] + nums[4] = 0 + 1 + (-1) = 0.
+nums[0] + nums[3] + nums[4] = (-1) + 2 + (-1) = 0.
+The distinct triplets are [-1,0,1] and [-1,-1,2].
+Notice that the order of the output and the order of the triplets does not matter.
+Example 2:
+Input: nums = [0,1,1]
+Output: []
+Explanation: The only possible triplet does not sum up to 0.
+Example 3:
+Input: nums = [0,0,0]
+Output: [[0,0,0]]
+Explanation: The only possible triplet sums up to 0.
+Constraints:
+3 &lt;= nums.length &lt;= 3000
+-10^5 &lt;= nums[i] &lt;= 10^5</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def threeSum(self, nums: List[int]) -&gt; List[List[int]]:        
+        n = len(nums)
+        ans = []
+        nums.sort()        
+        for i in range(n):      
+            if nums[i] &gt; 0:
+                break
+            if i &gt; 0 and nums[i] == nums[i-1]:
+                continue
+            l, r = i + 1, n - 1
+            while l &lt; r:
+                total = nums[i] + nums[l] + nums[r]
+                if total == 0:
+                    ans.append([nums[i], nums[l], nums[r]])
+                    l += 1
+                    r -= 1
+                    while l &lt; n - 1 and nums[l] == nums[l-1]:
+                        l += 1
+                elif total &lt; 0:
+                    l += 1
+                else:
+                    r -= 1
+        return ans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">class Solution:
+    def threeSum(self, nums: List[int]) -&gt; List[List[int]]:        </t>
+  </si>
+  <si>
+    <t>Given an integer array nums sorted in non-decreasing order, remove some duplicates in-place such that each unique element appears at most twice. The relative order of the elements should be kept the same.
+Since it is impossible to change the length of the array in some languages, you must instead have the result be placed in the first part of the array nums. More formally, if there are k elements after removing the duplicates, then the first k elements of nums should hold the final result. It does not matter what you leave beyond the first k elements.
+Return k after placing the final result in the first k slots of nums.
+Do not allocate extra space for another array. You must do this by modifying the input array in-place with O(1) extra memory.
+Custom Judge:
+The judge will test your solution with the following code:
+int[] nums = [...]; // Input array
+int[] expectedNums = [...]; // The expected answer with correct length
+int k = removeDuplicates(nums); // Calls your implementation
+assert k == expectedNums.length;
+for (int i = 0; i &lt; k; i++) {
+    assert nums[i] == expectedNums[i];
+}
+If all assertions pass, then your solution will be accepted.
+Example 1:
+Input: nums = [1,1,1,2,2,3]
+Output: 5, nums = [1,1,2,2,3,_]
+Explanation: Your function should return k = 5, with the first five elements of nums being 1, 1, 2, 2 and 3 respectively.
+It does not matter what you leave beyond the returned k (hence they are underscores).
+Example 2:
+Input: nums = [0,0,1,1,1,1,2,3,3]
+Output: 7, nums = [0,0,1,1,2,3,3,_,_]
+Explanation: Your function should return k = 7, with the first seven elements of nums being 0, 0, 1, 1, 2, 3 and 3 respectively.
+It does not matter what you leave beyond the returned k (hence they are underscores).
+Constraints:
+1 &lt;= nums.length &lt;= 3 * 104
+-104 &lt;= nums[i] &lt;= 104
+nums is sorted in non-decreasing order.</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def removeDuplicates(self, nums: List[int]) -&gt; int:</t>
+  </si>
+  <si>
+    <t>Array
+Two Pointers</t>
+  </si>
+  <si>
+    <t>Array
+Two Pointers
+Sorting</t>
+  </si>
+  <si>
+    <t>Given n non-negative integers representing an elevation map where the width of each bar is 1, compute how much water it can trap after raining.
+Example 1:
+Input: height = [0,1,0,2,1,0,1,3,2,1,2,1]
+Output: 6
+Explanation: The above elevation map (black section) is represented by array [0,1,0,2,1,0,1,3,2,1,2,1]. In this case, 6 units of rain water (blue section) are being trapped.
+Example 2:
+Input: height = [4,2,0,3,2,5]
+Output: 9
+Constraints:
+n == height.length
+1 &lt;= n &lt;= 2 * 10^4
+0 &lt;= height[i] &lt;= 10^5</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def trap(self, height: List[int]) -&gt; int:</t>
+  </si>
+  <si>
+    <t>Array
+Two Pointers
+Dynamic Programming</t>
+  </si>
+  <si>
+    <t>Given a string s, find the length of the longest substring without duplicate characters.
+Example 1:
+Input: s = "abcabcbb"
+Output: 3
+Explanation: The answer is "abc", with the length of 3.
+Example 2:
+Input: s = "bbbbb"
+Output: 1
+Explanation: The answer is "b", with the length of 1.
+Example 3:
+Input: s = "pwwkew"
+Output: 3
+Explanation: The answer is "wke", with the length of 3.
+Notice that the answer must be a substring, "pwke" is a subsequence and not a substring.
+Constraints:
+0 &lt;= s.length &lt;= 5 * 10^4
+s consists of English letters, digits, symbols and spaces.</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def lengthOfLongestSubstring(self, s: str) -&gt; int:</t>
+  </si>
+  <si>
+    <t>Hash Table
+String
+Sliding Window</t>
+  </si>
+  <si>
+    <t>Given two strings s and t of lengths m and n respectively, return the minimum window substring of s such that every character in t (including duplicates) is included in the window. If there is no such substring, return the empty string "".
+The testcases will be generated such that the answer is unique.
+Example 1:
+Input: s = "ADOBECODEBANC", t = "ABC"
+Output: "BANC"
+Explanation: The minimum window substring "BANC" includes 'A', 'B', and 'C' from string t.
+Example 2:
+Input: s = "a", t = "a"
+Output: "a"
+Explanation: The entire string s is the minimum window.
+Example 3:
+Input: s = "a", t = "aa"
+Output: ""
+Explanation: Both 'a's from t must be included in the window.
+Since the largest window of s only has one 'a', return empty string.
+Constraints:
+m == s.length
+n == t.length
+1 &lt;= m, n &lt;= 10^5
+s and t consist of uppercase and lowercase English letters.</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def minWindow(self, s: str, t: str) -&gt; str:</t>
+  </si>
+  <si>
+    <t>ou are given an array of integers nums, there is a sliding window of size k which is moving from the very left of the array to the very right. You can only see the k numbers in the window. Each time the sliding window moves right by one position.
+Return the max sliding window.
+Example 1:
+Input: nums = [1,3,-1,-3,5,3,6,7], k = 3
+Output: [3,3,5,5,6,7]
+Explanation: 
+Window position                Max
+---------------               -----
+[1  3  -1] -3  5  3  6  7       3
+ 1 [3  -1  -3] 5  3  6  7       3
+ 1  3 [-1  -3  5] 3  6  7       5
+ 1  3  -1 [-3  5  3] 6  7       5
+ 1  3  -1  -3 [5  3  6] 7       6
+ 1  3  -1  -3  5 [3  6  7]      7
+Example 2:
+Input: nums = [1], k = 1
+Output: [1]
+Constraints:
+1 &lt;= nums.length &lt;= 10^5
+-10^4 &lt;= nums[i] &lt;= 10^4
+1 &lt;= k &lt;= nums.length</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def maxSlidingWindow(self, nums: List[int], k: int) -&gt; List[int]:</t>
+  </si>
+  <si>
+    <t>Array
+Queue
+Sliding Window</t>
+  </si>
+  <si>
+    <t>Given two strings s1 and s2, return true if s2 contains a permutation of s1, or false otherwise.
+In other words, return true if one of s1's permutations is the substring of s2.
+Example 1:
+Input: s1 = "ab", s2 = "eidbaooo"
+Output: true
+Explanation: s2 contains one permutation of s1 ("ba").
+Example 2:
+Input: s1 = "ab", s2 = "eidboaoo"
+Output: false
+Constraints:
+1 &lt;= s1.length, s2.length &lt;= 10^4
+s1 and s2 consist of lowercase English letters.</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def checkInclusion(self, s1: str, s2: str) -&gt; bool:
+        if len(s2) &lt; len(s1):
+            return False
+        if s2==s1:
+            return True
+        s1_counts = [0]*26
+        s2_counts = [0]*26 
+        for i in range(len(s1)):
+            s1_counts[ord(s1[i])-97]+=1
+            s2_counts[ord(s2[i])-97]+=1
+        l=0
+        for c in s2[len(s1):]:
+            if s2_counts==s1_counts:
+                return True
+            s2_counts[ord(s2[l])-97]-=1
+            l+=1
+            s2_counts[ord(c)-97]+=1
+        return s2_counts==s1_counts</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def checkInclusion(self, s1: str, s2: str) -&gt; bool:</t>
+  </si>
+  <si>
+    <t>Hash Table
+Two Pointers
+String
+Sliding Window</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def reverseBits(self, n: int) -&gt; int:
+        return int(bin(n)[2:].zfill(32)[::-1], 2)</t>
+  </si>
+  <si>
+    <t>Reverse bits of a given 32 bits unsigned integer.
+Example 1:
+Input: n = 00000010100101000001111010011100
+Output:    964176192 (00111001011110000010100101000000)
+Explanation: The input binary string 00000010100101000001111010011100 represents the unsigned integer 43261596, so return 964176192 which its binary representation is 00111001011110000010100101000000.
+Example 2:
+Input: n = 11111111111111111111111111111101
+Output:   3221225471 (10111111111111111111111111111111)
+Explanation: The input binary string 11111111111111111111111111111101 represents the unsigned integer 4294967293, so return 3221225471 which its binary representation is 10111111111111111111111111111111.
+Constraints:
+The input must be a binary string of length 32</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def reverseBits(self, n: int) -&gt; int:</t>
+  </si>
+  <si>
+    <t>Divide and Conquer
+Bit Manipulation</t>
+  </si>
+  <si>
+    <t>Given an integer array nums, return the maximum result of nums[i] XOR nums[j], where 0 &lt;= i &lt;= j &lt; n.
+Example 1:
+Input: nums = [3,10,5,25,2,8]
+Output: 28
+Explanation: The maximum result is 5 XOR 25 = 28.
+Example 2:
+Input: nums = [14,70,53,83,49,91,36,80,92,51,66,70]
+Output: 127
+Constraints:
+1 &lt;= nums.length &lt;= 2 * 10^5
+0 &lt;= nums[i] &lt;= 2^31 - 1</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def findMaximumXOR(self, nums: List[int]) -&gt; int:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Array
+Hash Table
+Bit Manipulation
+</t>
+  </si>
+  <si>
+    <t>Merge K Sorted Lists</t>
+  </si>
+  <si>
+    <t>You are given an array of k linked-lists lists, each linked-list is sorted in ascending order.
+Merge all the linked-lists into one sorted linked-list and return it.
+Example 1:
+Input: lists = [[1,4,5],[1,3,4],[2,6]]
+Output: [1,1,2,3,4,4,5,6]
+Explanation: The linked-lists are:
+[
+  1-&gt;4-&gt;5,
+  1-&gt;3-&gt;4,
+  2-&gt;6
+]
+merging them into one sorted list:
+1-&gt;1-&gt;2-&gt;3-&gt;4-&gt;4-&gt;5-&gt;6
+Example 2:
+Input: lists = []
+Output: []
+Example 3:
+Input: lists = [[]]
+Output: []
+Constraints:
+k == lists.length
+0 &lt;= k &lt;= 10^4
+0 &lt;= lists[i].length &lt;= 500
+-104 &lt;= lists[i][j] &lt;= 10^4
+lists[i] is sorted in ascending order.
+The sum of lists[i].length will not exceed 10^4.</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def mergeKLists(self, lists: List[Optional[ListNode]]) -&gt; Optional[ListNode]:
+        if not lists:
+            return None
+        nodes = []
+        for lis in lists:
+            while lis:
+                nodes.append(lis.val)
+                lis = lis.next
+        head = ListNode(0)
+        node = head
+        for node_val in sorted(nodes):
+            newnode = ListNode(node_val)
+            node.next = newnode
+            node = node.next
+        return head.next</t>
+  </si>
+  <si>
+    <t>Linked List
+Divide and Conquer
+Merge Sort</t>
+  </si>
+  <si>
+    <t>Reverse Nodes in k-Group</t>
+  </si>
+  <si>
+    <t>Given the head of a linked list, reverse the nodes of the list k at a time, and return the modified list.
+k is a positive integer and is less than or equal to the length of the linked list. If the number of nodes is not a multiple of k then left-out nodes, in the end, should remain as it is.
+You may not alter the values in the list's nodes, only nodes themselves may be changed.
+Example 1:
+Input: head = [1,2,3,4,5], k = 2
+Output: [2,1,4,3,5]
+Example 2:
+Input: head = [1,2,3,4,5], k = 3
+Output: [3,2,1,4,5]
+Constraints:
+The number of nodes in the list is n.
+1 &lt;= k &lt;= n &lt;= 5000
+0 &lt;= Node.val &lt;= 1000</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def reverseKGroup(self, head: Optional[ListNode], k: int) -&gt; Optional[ListNode]:
+        def rev(head):
+            if head.next == None: return head, head
+            nh, nt = rev(head.next)
+            nt.next = head
+            head.next = None
+            return nh, head
+        def rev_k(head, k):
+            if head == None: return None
+            cnt = 1
+            prev_head = head
+            cur = head
+            while cur.next != None and cnt &lt; k:
+                cur = cur.next
+                cnt += 1
+            if cnt &lt; k:
+                return prev_head
+            tmp = cur.next
+            cur.next = None
+            ret, new_tail = rev(prev_head)
+            new_tail.next = rev_k(tmp, k)
+            return ret
+        return rev_k(head,k)</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def reverseKGroup(self, head: Optional[ListNode], k: int) -&gt; Optional[ListNode]:</t>
+  </si>
+  <si>
+    <t>Linked List
+Recursion</t>
+  </si>
+  <si>
+    <t>Flatten Binary Tree to Linked List</t>
+  </si>
+  <si>
+    <t>Given the root of a binary tree, flatten the tree into a "linked list":
+The "linked list" should use the same TreeNode class where the right child pointer points to the next node in the list and the left child pointer is always null.
+The "linked list" should be in the same order as a pre-order traversal of the binary tree.
+Example 1:
+Input: root = [1,2,5,3,4,null,6]
+Output: [1,null,2,null,3,null,4,null,5,null,6]
+Example 2:
+Input: root = []
+Output: []
+Example 3:
+Input: root = [0]
+Output: [0]
+Constraints:
+The number of nodes in the tree is in the range [0, 2000].
+-100 &lt;= Node.val &lt;= 100</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def flatten(self, root: Optional[TreeNode]) -&gt; None:
+        """
+        Do not return anything, modify root in-place instead.
+        """
+        if root is None:
+            return
+        self.flatten(root.left)
+        self.flatten(root.right)
+        left = root.left
+        right = root.right
+        root.left = None
+        root.right = left
+        p = root
+        while p.right is not None:
+            p = p.right
+        p.right = right</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def flatten(self, root: Optional[TreeNode]) -&gt; None:
+        """
+        Do not return anything, modify root in-place instead.
+        """</t>
+  </si>
+  <si>
+    <t>Linked List
+Depth-First Search
+Binary Tree</t>
+  </si>
+  <si>
+    <t>Binary Tree Maximum Path Sum</t>
+  </si>
+  <si>
+    <t>A path in a binary tree is a sequence of nodes where each pair of adjacent nodes in the sequence has an edge connecting them. A node can only appear in the sequence at most once. Note that the path does not need to pass through the root.
+The path sum of a path is the sum of the node's values in the path.
+Given the root of a binary tree, return the maximum path sum of any non-empty path.
+Example 1:
+Input: root = [1,2,3]
+Output: 6
+Explanation: The optimal path is 2 -&gt; 1 -&gt; 3 with a path sum of 2 + 1 + 3 = 6.
+Example 2:
+Input: root = [-10,9,20,null,null,15,7]
+Output: 42
+Explanation: The optimal path is 15 -&gt; 20 -&gt; 7 with a path sum of 15 + 20 + 7 = 42.
+Constraints:
+The number of nodes in the tree is in the range [1, 3 * 10^4].
+-1000 &lt;= Node.val &lt;= 1000</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def maxPathSum(self, root: Optional[TreeNode]) -&gt; int:
+        global max_node
+        max_node=-float("inf")
+        def find(root: Optional[TreeNode],max_path_total,path_sum=0):
+            if root is None:
+                return 0,max_path_total
+            global max_node
+            if root.val&gt;max_node:
+                max_node=root.val
+            path_sum_l,max_path_total=find(root.left,max_path_total)
+            path_sum_r,max_path_total=find(root.right,max_path_total)
+            path_sum_l_r=max(max(path_sum_r,path_sum_l)+root.val,root.val)
+            path_total=path_sum_l+path_sum_r+root.val
+            if max_path_total&lt;path_total:
+                max_path_total=path_total
+            if path_sum_l_r&gt;max_path_total:
+                max_path_total=path_sum_l_r
+            return path_sum_l_r,max_path_total
+        r=find(root,-float("inf"))
+        return r[1]</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def maxPathSum(self, root: Optional[TreeNode]) -&gt; int:</t>
+  </si>
+  <si>
+    <t>Dynamic Programming
+Depth-First Search
+Binary Tree</t>
+  </si>
+  <si>
+    <t>Binary Tree Cameras</t>
+  </si>
+  <si>
+    <t>You are given the root of a binary tree. We install cameras on the tree nodes where each camera at a node can monitor its parent, itself, and its immediate children.
+Return the minimum number of cameras needed to monitor all nodes of the tree.
+Example 1:
+Input: root = [0,0,null,0,0]
+Output: 1
+Example 2:
+Input: root = [0,0,null,0,null,0,null,null,0]
+Output: 2
+Constraints:
+The number of nodes in the tree is in the range [1, 1000].
+Node.val == 0</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def minCameraCover(self, root: Optional[TreeNode]) -&gt; int:</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def minCameraCover(self, root: Optional[TreeNode]) -&gt; int:
+        self.cameras = 0
+        def dfs(node):
+            if not node:
+                return 1
+            left = dfs(node.left)
+            right = dfs(node.right)
+            if left == 0 or right == 0:
+                self.cameras += 1
+                return 2
+            if left == 2 or right == 2:
+                return 1
+            return 0
+        if dfs(root) == 0:
+            self.cameras += 1
+        return self.cameras</t>
+  </si>
+  <si>
+    <t>Vertical Order Traversal of a Binary Tree</t>
+  </si>
+  <si>
+    <t>Given the root of a binary tree, calculate the vertical order traversal of the binary tree.
+For each node at position (row, col), its left and right children will be at positions (row + 1, col - 1) and (row + 1, col + 1) respectively. The root of the tree is at (0, 0).
+The vertical order traversal of a binary tree is a list of top-to-bottom orderings for each column index starting from the leftmost column and ending on the rightmost column. There may be multiple nodes in the same row and same column. In such a case, sort these nodes by their values.
+Return the vertical order traversal of the binary tree.
+Example 1:
+Input: root = [3,9,20,null,null,15,7]
+Output: [[9],[3,15],[20],[7]]
+Explanation:
+Column -1: Only node 9 is in this column.
+Column 0: Nodes 3 and 15 are in this column in that order from top to bottom.
+Column 1: Only node 20 is in this column.
+Column 2: Only node 7 is in this column.
+Example 2:
+Input: root = [1,2,3,4,5,6,7]
+Output: [[4],[2],[1,5,6],[3],[7]]
+Explanation:
+Column -2: Only node 4 is in this column.
+Column -1: Only node 2 is in this column.
+Column 0: Nodes 1, 5, and 6 are in this column.
+          1 is at the top, so it comes first.
+          5 and 6 are at the same position (2, 0), so we order them by their value, 5 before 6.
+Column 1: Only node 3 is in this column.
+Column 2: Only node 7 is in this column.
+Example 3:
+Input: root = [1,2,3,4,6,5,7]
+Output: [[4],[2],[1,5,6],[3],[7]]
+Explanation:
+This case is the exact same as example 2, but with nodes 5 and 6 swapped.
+Note that the solution remains the same since 5 and 6 are in the same location and should be ordered by their values.
+Constraints:
+The number of nodes in the tree is in the range [1, 1000].
+0 &lt;= Node.val &lt;= 1000</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def verticalTraversal(self, root: Optional[TreeNode]) -&gt; List[List[int]]:</t>
+  </si>
+  <si>
+    <t>Hash Table
+Depth-First Search
+Breadth-First Search
+Binary Tree</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def verticalTraversal(self, root: Optional[TreeNode]) -&gt; List[List[int]]:
+        res = {}
+        def visit(node, row, col):
+            if not node:
+                return
+            if col not in res.keys():
+                res[col] = [(row, node.val)]
+            else:
+                res[col].append((row, node.val))
+            visit(node.left, row+1, col-1)
+            visit(node.right, row+1, col+1)
+        visit(root, 0, 0)
+        # print(res)
+        sorted_keys = sorted(res.keys())
+        output = []
+        for key in sorted_keys:
+            sorted_values = sorted(res[key], key=lambda x: (x[0], x[1]))
+            output.append([v[1] for v in sorted_values])
+        return output</t>
+  </si>
+  <si>
+    <t>Recover a Tree from PreOrder Traversal</t>
+  </si>
+  <si>
+    <t>We run a preorder depth-first search (DFS) on the root of a binary tree.
+At each node in this traversal, we output D dashes (where D is the depth of this node), then we output the value of this node.  If the depth of a node is D, the depth of its immediate child is D + 1.  The depth of the root node is 0.
+If a node has only one child, that child is guaranteed to be the left child.
+Given the output traversal of this traversal, recover the tree and return its root.
+Example 1:
+Input: traversal = "1-2--3--4-5--6--7"
+Output: [1,2,5,3,4,6,7]
+Example 2:
+Input: traversal = "1-2--3---4-5--6---7"
+Output: [1,2,5,3,null,6,null,4,null,7]
+Example 3:
+Input: traversal = "1-401--349---90--88"
+Output: [1,401,null,349,88,90]
+Constraints:
+The number of nodes in the original tree is in the range [1, 1000].
+1 &lt;= Node.val &lt;= 109</t>
+  </si>
+  <si>
+    <t>Depth-First Search
+Binary Tree</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def recoverFromPreorder(self, traversal: str) -&gt; Optional[TreeNode]:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">class Solution:
+    def recoverFromPreorder(self, traversal: str) -&gt; Optional[TreeNode]:
+        nodes = [(len(node[1]), int(node[2])) for node in re.findall("((-*)(\d+))", traversal)][::-1]
+        def makeTree(depth): 
+            if not nodes or depth != nodes[-1][0]: return None 
+            node = TreeNode(nodes.pop()[1])
+            node.left = makeTree(depth + 1) 
+            node.right = makeTree(depth + 1)
+            return node
+        return makeTree(0) </t>
   </si>
 </sst>
 </file>
@@ -2627,7 +3917,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="56" customWidth="1"/>
@@ -2652,7 +3942,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="360" x14ac:dyDescent="0.3">
@@ -2663,7 +3953,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
@@ -2672,7 +3962,7 @@
         <v>7</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="403.2" x14ac:dyDescent="0.3">
@@ -2683,7 +3973,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -2692,7 +3982,7 @@
         <v>9</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2703,7 +3993,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
@@ -2712,7 +4002,7 @@
         <v>12</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2723,7 +4013,7 @@
         <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
@@ -2732,7 +4022,7 @@
         <v>14</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="388.8" x14ac:dyDescent="0.3">
@@ -2743,16 +4033,16 @@
         <v>15</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2763,16 +4053,16 @@
         <v>16</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2783,7 +4073,7 @@
         <v>17</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -2792,7 +4082,7 @@
         <v>18</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2803,7 +4093,7 @@
         <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D9" t="s">
         <v>6</v>
@@ -2812,7 +4102,7 @@
         <v>20</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2823,16 +4113,16 @@
         <v>21</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
@@ -2843,7 +4133,7 @@
         <v>22</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>6</v>
@@ -2852,7 +4142,7 @@
         <v>23</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2863,7 +4153,7 @@
         <v>24</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
@@ -2872,7 +4162,7 @@
         <v>25</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
@@ -2883,7 +4173,7 @@
         <v>26</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>6</v>
@@ -2892,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2903,16 +4193,16 @@
         <v>28</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="D14" t="s">
         <v>6</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
@@ -2923,7 +4213,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
@@ -2932,7 +4222,7 @@
         <v>30</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="345.6" x14ac:dyDescent="0.3">
@@ -2943,7 +4233,7 @@
         <v>31</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
@@ -2952,10 +4242,10 @@
         <v>32</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="403.2" x14ac:dyDescent="0.3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2963,7 +4253,7 @@
         <v>33</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="D17" t="s">
         <v>6</v>
@@ -2972,10 +4262,10 @@
         <v>34</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2983,7 +4273,7 @@
         <v>35</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
@@ -2992,10 +4282,10 @@
         <v>36</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3003,7 +4293,7 @@
         <v>37</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
@@ -3012,10 +4302,10 @@
         <v>38</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3023,7 +4313,7 @@
         <v>39</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="D20" t="s">
         <v>6</v>
@@ -3032,10 +4322,10 @@
         <v>40</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -3043,7 +4333,7 @@
         <v>41</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>6</v>
@@ -3052,10 +4342,10 @@
         <v>42</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -3063,7 +4353,7 @@
         <v>43</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
@@ -3072,10 +4362,10 @@
         <v>44</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -3083,7 +4373,7 @@
         <v>45</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
@@ -3092,10 +4382,10 @@
         <v>46</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -3103,7 +4393,7 @@
         <v>47</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
@@ -3112,7 +4402,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:6" s="9" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" s="9" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A25" s="9">
         <v>24</v>
       </c>
@@ -3120,7 +4410,7 @@
         <v>49</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>140</v>
+        <v>124</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>6</v>
@@ -3129,7 +4419,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -3137,7 +4427,7 @@
         <v>51</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
@@ -3146,7 +4436,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -3154,7 +4444,7 @@
         <v>53</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
@@ -3163,7 +4453,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="403.2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -3171,7 +4461,7 @@
         <v>33</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="D28" t="s">
         <v>6</v>
@@ -3180,7 +4470,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3188,7 +4478,7 @@
         <v>55</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
@@ -3197,7 +4487,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -3205,7 +4495,7 @@
         <v>57</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
@@ -3214,185 +4504,606 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" t="s">
         <v>59</v>
       </c>
-      <c r="C31" t="s">
-        <v>60</v>
+      <c r="C31" s="1" t="s">
+        <v>173</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="E31" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>61</v>
-      </c>
-      <c r="C32" t="s">
-        <v>62</v>
+        <v>60</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>176</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="331.2" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="360" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>64</v>
-      </c>
-      <c r="C33" t="s">
-        <v>65</v>
+        <v>62</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>180</v>
       </c>
       <c r="D33" t="s">
         <v>6</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>67</v>
-      </c>
-      <c r="C34" t="s">
-        <v>68</v>
+        <v>64</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>183</v>
       </c>
       <c r="D34" t="s">
         <v>11</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="360" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>70</v>
-      </c>
-      <c r="C35" t="s">
-        <v>71</v>
+        <v>66</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>186</v>
       </c>
       <c r="D35" t="s">
         <v>6</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="216" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>73</v>
-      </c>
-      <c r="C36" t="s">
-        <v>74</v>
+        <v>68</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>188</v>
       </c>
       <c r="D36" t="s">
         <v>6</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
-      </c>
-      <c r="C37" t="s">
-        <v>77</v>
+        <v>70</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>191</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="E37" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>78</v>
-      </c>
-      <c r="C38" t="s">
-        <v>79</v>
+        <v>71</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>196</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>195</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>81</v>
-      </c>
-      <c r="C39" t="s">
-        <v>82</v>
+        <v>72</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>199</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>84</v>
-      </c>
-      <c r="C40" t="s">
-        <v>85</v>
+        <v>202</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>203</v>
       </c>
       <c r="D40" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+        <v>204</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>87</v>
-      </c>
-      <c r="C41" t="s">
-        <v>88</v>
+        <v>206</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>207</v>
       </c>
       <c r="D41" t="s">
         <v>6</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>89</v>
+        <v>208</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="403.2" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>211</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="D42" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>216</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D43" t="s">
+        <v>6</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>221</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="D44" t="s">
+        <v>6</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>225</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D45" t="s">
+        <v>6</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>230</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="D46" t="s">
+        <v>6</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C0B5B2B-B8E4-4AD0-AF1F-F0B32BC330F3}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="23.44140625" customWidth="1"/>
+    <col min="5" max="5" width="35.44140625" customWidth="1"/>
+    <col min="6" max="6" width="35.109375" customWidth="1"/>
+    <col min="7" max="7" width="32.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F1" t="s">
+        <v>132</v>
+      </c>
+      <c r="G1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>157</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>168</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="D9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
included binary tree and linked list questions
</commit_message>
<xml_diff>
--- a/temp_benchmark_data.xlsx
+++ b/temp_benchmark_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\megha\Managing data for minor\Major\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5243A763-1814-4BBE-ACD8-333DA9AA6175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C354E79-6851-4270-905D-C7641EBDDC8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2688,32 +2688,6 @@
   </si>
   <si>
     <t>class Solution:
-    def reverseKGroup(self, head: Optional[ListNode], k: int) -&gt; Optional[ListNode]:
-        def rev(head):
-            if head.next == None: return head, head
-            nh, nt = rev(head.next)
-            nt.next = head
-            head.next = None
-            return nh, head
-        def rev_k(head, k):
-            if head == None: return None
-            cnt = 1
-            prev_head = head
-            cur = head
-            while cur.next != None and cnt &lt; k:
-                cur = cur.next
-                cnt += 1
-            if cnt &lt; k:
-                return prev_head
-            tmp = cur.next
-            cur.next = None
-            ret, new_tail = rev(prev_head)
-            new_tail.next = rev_k(tmp, k)
-            return ret
-        return rev_k(head,k)</t>
-  </si>
-  <si>
-    <t>class Solution:
     def reverseKGroup(self, head: Optional[ListNode], k: int) -&gt; Optional[ListNode]:</t>
   </si>
   <si>
@@ -3047,6 +3021,36 @@
   <si>
     <t>class Solution:
     def maxArea(self, height: List[int]) -&gt; int:</t>
+  </si>
+  <si>
+    <t>class Solution:
+    def reverseKGroup(self, head: Optional[ListNode], k: int) -&gt; Optional[ListNode]:
+        dummy = ListNode()
+        dummy.next = head
+        prev_g_tail = dummy 
+        curr = head
+        while curr:
+            curr_g_head = curr
+            prev = None
+            for _ in range(k):
+                if curr:
+                    prev = curr
+                    curr = curr.next
+                else:
+                    return dummy.next
+            next_g_head = curr
+            curr_g_tail = prev
+            prev = next_g_head
+            curr = curr_g_head
+            for _ in range(k):
+                tmp = curr.next
+                curr.next = prev
+                prev = curr
+                curr = tmp
+            prev_g_tail.next = curr_g_tail
+            prev_g_tail = curr_g_head
+            curr = next_g_head
+        return dummy.next</t>
   </si>
 </sst>
 </file>
@@ -4436,7 +4440,7 @@
         <v>48</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="25" spans="1:7" s="9" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
@@ -4456,7 +4460,7 @@
         <v>50</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
@@ -4476,7 +4480,7 @@
         <v>52</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
@@ -4496,7 +4500,7 @@
         <v>54</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="403.2" x14ac:dyDescent="0.3">
@@ -4536,7 +4540,7 @@
         <v>56</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
@@ -4556,7 +4560,7 @@
         <v>58</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="31" spans="1:7" s="11" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
@@ -4590,7 +4594,7 @@
         <v>60</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
@@ -4682,7 +4686,7 @@
         <v>68</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D36" t="s">
         <v>6</v>
@@ -4789,7 +4793,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="403.2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -4803,13 +4807,13 @@
         <v>6</v>
       </c>
       <c r="E41" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="F41" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="G41" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="403.2" x14ac:dyDescent="0.3">
@@ -4817,22 +4821,22 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
+        <v>208</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>210</v>
       </c>
       <c r="D42" t="s">
         <v>11</v>
       </c>
       <c r="E42" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="G42" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
@@ -4840,22 +4844,22 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
+        <v>213</v>
+      </c>
+      <c r="C43" s="1" t="s">
         <v>214</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>215</v>
       </c>
       <c r="D43" t="s">
         <v>6</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="G43" s="1" t="s">
         <v>217</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="316.8" x14ac:dyDescent="0.3">
@@ -4863,22 +4867,22 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
+        <v>218</v>
+      </c>
+      <c r="C44" s="1" t="s">
         <v>219</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>220</v>
       </c>
       <c r="D44" t="s">
         <v>6</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
@@ -4886,22 +4890,22 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
+        <v>222</v>
+      </c>
+      <c r="C45" s="1" t="s">
         <v>223</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>224</v>
       </c>
       <c r="D45" t="s">
         <v>6</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F45" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="G45" s="1" t="s">
         <v>225</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
@@ -4909,22 +4913,22 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
+        <v>227</v>
+      </c>
+      <c r="C46" s="1" t="s">
         <v>228</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>229</v>
       </c>
       <c r="D46" t="s">
         <v>6</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>